<commit_message>
Add Texas dental suppliers 2026-06-12
</commit_message>
<xml_diff>
--- a/output/Texas_Dental_Suppliers.xlsx
+++ b/output/Texas_Dental_Suppliers.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>64%</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -657,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -666,14 +666,16 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="36" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="32" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -718,45 +720,55 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Email *</t>
+          <t>Email 1 *</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
+          <t>Email 2 *</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Contact Form *</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
           <t>Decision Maker *</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Title *</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>What They Sell *</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>Territory *</t>
         </is>
       </c>
-      <c r="K3" s="8" t="inlineStr">
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>Brands Carried *</t>
         </is>
       </c>
-      <c r="L3" s="8" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Years in Business *</t>
         </is>
       </c>
-      <c r="M3" s="8" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>LinkedIn *</t>
         </is>
       </c>
-      <c r="N3" s="8" t="inlineStr">
+      <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Social Media *</t>
         </is>
@@ -831,6 +843,16 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="11" t="n">
@@ -838,7 +860,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Martinez Dentalcraft &amp; Equipment Inc</t>
+          <t>Reliable Dental Supply &amp; Service Company</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -848,17 +870,17 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>(817) 926-1247</t>
+          <t>(817) 927-5909</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://martinezdentalcraft.com/</t>
+          <t>http://www.reliabledental.com/</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>lindab@martinezdentalcraft.com</t>
+          <t>rds@reliabledental.com</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
@@ -873,7 +895,7 @@
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>Dental Equipment, Dental Software, Sterilisation, Dental Furniture</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J5" s="12" t="inlineStr">
@@ -883,12 +905,12 @@
       </c>
       <c r="K5" s="12" t="inlineStr">
         <is>
-          <t>3M</t>
+          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="M5" s="12" t="inlineStr">
@@ -897,6 +919,16 @@
         </is>
       </c>
       <c r="N5" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O5" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P5" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -908,27 +940,27 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Reliable Dental Supply &amp; Service Company</t>
+          <t>Lone Star Dental Corp</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Fort Worth</t>
+          <t>Arlington</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>(817) 927-5909</t>
+          <t>(682) 564-0772</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>http://www.reliabledental.com/</t>
+          <t>https://www.lonestardentalcorp.com/</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>lonestardentalcorp.4@gmail.com</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -943,22 +975,22 @@
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Equipment, Dental Supplies, Sterilisation, Dental Furniture</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas, Nationwide</t>
         </is>
       </c>
       <c r="M6" s="10" t="inlineStr">
@@ -968,7 +1000,17 @@
       </c>
       <c r="N6" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Since 1983</t>
+        </is>
+      </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t>Facebook, Google Business</t>
         </is>
       </c>
     </row>
@@ -978,27 +1020,27 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Garland Dental Equipment Services</t>
+          <t>Hewitt Dental Inc</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Garland</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>(214) 461-5618</t>
+          <t>(512) 873-8847</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://www.garlanddental.com/</t>
+          <t>http://www.hewittdental.com/</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>officemanager@hewittdental.com</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
@@ -1013,7 +1055,7 @@
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>Digital Dentistry, Repair &amp; Service</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
@@ -1023,20 +1065,30 @@
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Equipment, Orthodontic Supplies, Sterilisation, Dental Furniture</t>
         </is>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>KaVo, Midmark</t>
         </is>
       </c>
       <c r="N7" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O7" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P7" s="12" t="inlineStr">
         <is>
           <t>Facebook, Instagram</t>
         </is>
@@ -1048,32 +1100,32 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Midwest Dental Equipment &amp; Supplies</t>
+          <t>Martinez Dentalcraft &amp; Equipment Inc</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Fort Worth</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>(210) 981-2264</t>
+          <t>(817) 926-1247</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>https://midwestdental.com/san_antonio</t>
+          <t>https://martinezdentalcraft.com/</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>lindab@martinezdentalcraft.com</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>roym@martinezdentalcraft.com</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr">
@@ -1093,7 +1145,7 @@
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Equipment, Dental Software, Sterilisation, Dental Furniture</t>
         </is>
       </c>
       <c r="L8" s="10" t="inlineStr">
@@ -1103,10 +1155,20 @@
       </c>
       <c r="M8" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3M</t>
         </is>
       </c>
       <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P8" s="10" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1118,22 +1180,22 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Lone Star Dental Corp</t>
+          <t>Midwest Dental Equipment &amp; Supplies</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Arlington</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>(682) 564-0772</t>
+          <t>(210) 981-2264</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>https://www.lonestardentalcorp.com/</t>
+          <t>https://midwestdental.com/san_antonio</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -1153,12 +1215,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Dental Equipment, Dental Supplies, Sterilisation, Dental Furniture</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Texas, Nationwide</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -1168,7 +1230,7 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>Since 1983</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="M9" s="12" t="inlineStr">
@@ -1178,7 +1240,17 @@
       </c>
       <c r="N9" s="12" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P9" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1188,22 +1260,22 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>TM Global Equipment</t>
+          <t>Midwest Dental Houston, TX</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Garland</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>(800) 770-9234</t>
+          <t>(713) 955-7299</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>http://www.tmglobalequipment.com/</t>
+          <t>https://midwestdental.com/houston</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -1247,6 +1319,16 @@
         </is>
       </c>
       <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P10" s="10" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1258,27 +1340,27 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Dental Equipment Liquidators, Inc,</t>
+          <t>Capital Dental Equipment</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Hudson</t>
+          <t>New Braunfels</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>(727) 863-5500</t>
+          <t>(830) 730-0671</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>http://dentalequipment.com/</t>
+          <t>http://www.capitaldentalequipment.com/</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>jacobv@capitaldentalequipment.com</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -1293,32 +1375,42 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>Dental Equipment, Orthodontic Supplies, Sterilisation, Dental Furniture</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Texas, Nationwide</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>Dentsply, Patterson, Henry Schein, Sirona, KaVo</t>
+          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>Since 1998</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dentsply, Carestream, Midmark, A-dec, Belmont</t>
         </is>
       </c>
       <c r="N11" s="12" t="inlineStr">
         <is>
-          <t>Facebook, YouTube</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P11" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -1328,27 +1420,27 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Capital Dental Equipment</t>
+          <t>Midwest Dental</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>New Braunfels</t>
+          <t>Grand Prairie</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>(830) 730-0671</t>
+          <t>(817) 469-1929</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>http://www.capitaldentalequipment.com/</t>
+          <t>https://midwestdental.com/dallas_worth</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>jacobv@capitaldentalequipment.com</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -1363,7 +1455,7 @@
       </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
-          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J12" s="10" t="inlineStr">
@@ -1373,7 +1465,7 @@
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>Dentsply, Carestream, Midmark, A-dec, Belmont</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L12" s="10" t="inlineStr">
@@ -1387,6 +1479,16 @@
         </is>
       </c>
       <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P12" s="10" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1398,27 +1500,27 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>DFW Dental Supply</t>
+          <t>DuraPro Health – Dental Planet</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Garland</t>
+          <t>Wichita Falls</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>(800) 770-9234</t>
+          <t>(940) 766-5209</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>http://www.dfwdentalsupply.com/</t>
+          <t>https://www.duraprohealth.com/</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>sales@duraprohealth.com</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
@@ -1443,7 +1545,7 @@
       </c>
       <c r="K13" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Equipment, Dental Supplies, Sterilisation, Dental Furniture</t>
         </is>
       </c>
       <c r="L13" s="12" t="inlineStr">
@@ -1453,12 +1555,22 @@
       </c>
       <c r="M13" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Carestream, A-dec</t>
         </is>
       </c>
       <c r="N13" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="O13" s="12" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/DuraProHealth</t>
+        </is>
+      </c>
+      <c r="P13" s="12" t="inlineStr">
+        <is>
+          <t>Facebook, Instagram, Twitter/X, YouTube, Pinterest</t>
         </is>
       </c>
     </row>
@@ -1468,57 +1580,57 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Archer Dental</t>
+          <t>Burkhart Dental Supply - Dallas</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Plano</t>
+          <t>Irving</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>(972) 801-9750</t>
+          <t>(800) 324-4868</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>http://www.archerdental.com/</t>
+          <t>https://www.burkhartdental.com/</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Dylan@ArcherDental.com</t>
+          <t>practicesupportteam@burkhartdental.com</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Tech West</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
         <is>
-          <t>Dental Equipment, Sterilisation, Dental Furniture, Digital Dentistry</t>
+          <t>Burkhart Account</t>
         </is>
       </c>
       <c r="J14" s="10" t="inlineStr">
         <is>
-          <t>Texas, Nationwide</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t>KaVo, Midmark, A-dec</t>
+          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
         </is>
       </c>
       <c r="L14" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="M14" s="10" t="inlineStr">
@@ -1528,7 +1640,17 @@
       </c>
       <c r="N14" s="10" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O14" s="10" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/burkhart-dental-supply</t>
+        </is>
+      </c>
+      <c r="P14" s="10" t="inlineStr">
+        <is>
+          <t>Facebook, Twitter/X</t>
         </is>
       </c>
     </row>
@@ -1538,22 +1660,22 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Dental Health Products, Inc. (DHP)</t>
+          <t>Dental Equipment Liquidators, Inc,</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Sugar Land</t>
+          <t>Hudson</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>(800) 626-2163</t>
+          <t>(727) 863-5500</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>https://www.dhpsupply.com/</t>
+          <t>http://dentalequipment.com/</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -1568,37 +1690,47 @@
       </c>
       <c r="H15" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://www.dentalequipment.com/index.php?l=page_view&amp;p=contact_us</t>
         </is>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Dental Supplies, Orthodontic Supplies, Sterilisation, Dental Furniture</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>Texas, Southwest, Southeast</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
         <is>
-          <t>3M</t>
+          <t>Dental Equipment, Orthodontic Supplies, Sterilisation, Dental Furniture</t>
         </is>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas, Nationwide</t>
         </is>
       </c>
       <c r="M15" s="12" t="inlineStr">
         <is>
-          <t>linkedin.com/company/dhpsupply</t>
+          <t>Dentsply, Patterson, Henry Schein, Sirona, KaVo</t>
         </is>
       </c>
       <c r="N15" s="12" t="inlineStr">
         <is>
-          <t>Facebook, Instagram, Twitter/X, YouTube</t>
+          <t>Since 1998</t>
+        </is>
+      </c>
+      <c r="O15" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P15" s="12" t="inlineStr">
+        <is>
+          <t>Facebook, YouTube, Google Business</t>
         </is>
       </c>
     </row>
@@ -1608,27 +1740,27 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Midwest Dental</t>
+          <t>Dental Health Products, Inc. (DHP)</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Grand Prairie</t>
+          <t>Dallas</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>(817) 469-1929</t>
+          <t>(800) 528-4231</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>https://midwestdental.com/dallas_worth</t>
+          <t>https://www.dhpsupply.com/</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>support@dhpsupply.com</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -1653,22 +1785,32 @@
       </c>
       <c r="K16" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Supplies, Orthodontic Supplies, Sterilisation, Dental Furniture</t>
         </is>
       </c>
       <c r="L16" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas, Southwest, Southeast</t>
         </is>
       </c>
       <c r="M16" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3M</t>
         </is>
       </c>
       <c r="N16" s="10" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="O16" s="10" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/dhpsupply</t>
+        </is>
+      </c>
+      <c r="P16" s="10" t="inlineStr">
+        <is>
+          <t>Facebook, Instagram, Twitter/X, YouTube</t>
         </is>
       </c>
     </row>
@@ -1678,22 +1820,22 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Midwest Dental Houston, TX</t>
+          <t>The Device Doctor, LLC</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Burleson</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>(713) 955-7299</t>
+          <t>(800) 817-7491</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>https://midwestdental.com/houston</t>
+          <t>http://devicedoctor.dental/</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -1723,7 +1865,7 @@
       </c>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Equipment, Repair &amp; Service</t>
         </is>
       </c>
       <c r="L17" s="12" t="inlineStr">
@@ -1737,6 +1879,16 @@
         </is>
       </c>
       <c r="N17" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O17" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P17" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1748,27 +1900,27 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Hewitt Dental Inc</t>
+          <t>Edison Medical | Dental Implant USA</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>(512) 873-8847</t>
+          <t>(855) 807-8111</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>http://www.hewittdental.com/</t>
+          <t>https://edisonmed.com/</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>officemanager@hewittdental.com</t>
+          <t>info@edisonmed.com</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -1783,17 +1935,17 @@
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>Dental Equipment, Orthodontic Supplies, Sterilisation, Dental Furniture</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J18" s="10" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K18" s="10" t="inlineStr">
         <is>
-          <t>KaVo, Midmark</t>
+          <t>Digital Dentistry</t>
         </is>
       </c>
       <c r="L18" s="10" t="inlineStr">
@@ -1803,12 +1955,22 @@
       </c>
       <c r="M18" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Sirona</t>
         </is>
       </c>
       <c r="N18" s="10" t="inlineStr">
         <is>
-          <t>Facebook, Instagram</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O18" s="10" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/edisonmedical</t>
+        </is>
+      </c>
+      <c r="P18" s="10" t="inlineStr">
+        <is>
+          <t>Facebook, Instagram, Twitter/X, YouTube</t>
         </is>
       </c>
     </row>
@@ -1818,32 +1980,32 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>US Dental Depot - Dental Supplies</t>
+          <t>Archer Dental</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Boca Raton</t>
+          <t>Plano</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>(954) 874-6325</t>
+          <t>(972) 801-9750</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>http://www.usdentaldepot.com/</t>
+          <t>http://www.archerdental.com/</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>dylan@archerdental.com</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>james@archerdental.com</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
@@ -1853,32 +2015,42 @@
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Tech West</t>
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>VP</t>
         </is>
       </c>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Equipment, Sterilisation, Dental Furniture, Digital Dentistry</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas, Nationwide</t>
         </is>
       </c>
       <c r="M19" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>KaVo, Midmark, A-dec</t>
         </is>
       </c>
       <c r="N19" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="O19" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P19" s="12" t="inlineStr">
+        <is>
+          <t>YouTube</t>
         </is>
       </c>
     </row>
@@ -1888,22 +2060,22 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Dental Equipment Specialists</t>
+          <t>Midwest Dental Equipment &amp; Supply</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Crofton</t>
+          <t>Hewitt</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>(410) 257-2323</t>
+          <t>(800) 766-2025</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>http://desdental.com/</t>
+          <t>http://www.midwestdental.com/</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -1947,6 +2119,16 @@
         </is>
       </c>
       <c r="N20" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O20" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P20" s="10" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1958,22 +2140,22 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Burkhart Dental Supply - Dallas</t>
+          <t>Ross Orthodontic Equipment</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Irving</t>
+          <t>Midlothian</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>(800) 324-4868</t>
+          <t>(800) 247-4109</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>https://www.burkhartdental.com/</t>
+          <t>http://www.rossorthodontic.com/</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
@@ -1983,42 +2165,52 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>Burkhart Account</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>http://rossorthodontic.com/contact/</t>
         </is>
       </c>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J21" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K21" s="12" t="inlineStr">
+        <is>
+          <t>Orthodontic Supplies, Sterilisation, Repair &amp; Service</t>
+        </is>
+      </c>
+      <c r="L21" s="12" t="inlineStr">
+        <is>
           <t>Texas</t>
         </is>
       </c>
-      <c r="K21" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L21" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="M21" s="12" t="inlineStr">
         <is>
-          <t>linkedin.com/company/burkhart-dental-supply</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N21" s="12" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>Since 1982</t>
+        </is>
+      </c>
+      <c r="O21" s="12" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/ross-orthodontics</t>
+        </is>
+      </c>
+      <c r="P21" s="12" t="inlineStr">
+        <is>
+          <t>Facebook, Instagram, Twitter/X, Google Business</t>
         </is>
       </c>
     </row>
@@ -2028,22 +2220,22 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Houston Dental Supply</t>
+          <t>Handpiece Express</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>The Woodlands</t>
+          <t>Round Rock</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>(832) 844-5551</t>
+          <t>(800) 895-7111</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://www.myhandpiecerepair.com/</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -2058,7 +2250,7 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>https://www.myhandpiecerepair.com/contact-us/</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
@@ -2073,12 +2265,12 @@
       </c>
       <c r="K22" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Equipment, Repair &amp; Service</t>
         </is>
       </c>
       <c r="L22" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="M22" s="10" t="inlineStr">
@@ -2089,6 +2281,16 @@
       <c r="N22" s="10" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="O22" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P22" s="10" t="inlineStr">
+        <is>
+          <t>Facebook, Twitter/X, Pinterest, WhatsApp, Google Business</t>
         </is>
       </c>
     </row>
@@ -2098,27 +2300,27 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Benco Dental</t>
+          <t>Burkhart Dental Supply - Austin</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Flower Mound</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>(972) 355-1359</t>
+          <t>(877) 363-8717</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>https://www.benco.com/</t>
+          <t>http://www.burkhartdental.com/</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>practicesupportteam@burkhartdental.com</t>
         </is>
       </c>
       <c r="G23" s="12" t="inlineStr">
@@ -2133,22 +2335,22 @@
       </c>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>Dental Supplies, Digital Dentistry</t>
+          <t>Burkhart Account</t>
         </is>
       </c>
       <c r="J23" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="K23" s="12" t="inlineStr">
         <is>
-          <t>Ivoclar</t>
+          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
         </is>
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="M23" s="12" t="inlineStr">
@@ -2158,7 +2360,17 @@
       </c>
       <c r="N23" s="12" t="inlineStr">
         <is>
-          <t>Facebook, Instagram, Twitter/X, YouTube</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O23" s="12" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/burkhart-dental-supply</t>
+        </is>
+      </c>
+      <c r="P23" s="12" t="inlineStr">
+        <is>
+          <t>Facebook, Twitter/X</t>
         </is>
       </c>
     </row>
@@ -2168,27 +2380,27 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Dental Health Products, Inc. (DHP)</t>
+          <t>DFW Dental Supply</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Dallas</t>
+          <t>Garland</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>(800) 528-4231</t>
+          <t>(800) 770-9234</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>https://www.dhpsupply.com/</t>
+          <t>http://www.dfwdentalsupply.com/</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>sales@dfwdentalsupply.com</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -2203,32 +2415,42 @@
       </c>
       <c r="I24" s="10" t="inlineStr">
         <is>
-          <t>Dental Supplies, Orthodontic Supplies, Sterilisation, Dental Furniture</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>Texas, Southwest, Southeast</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
-          <t>3M</t>
+          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
         </is>
       </c>
       <c r="L24" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="M24" s="10" t="inlineStr">
         <is>
-          <t>linkedin.com/company/dhpsupply</t>
+          <t>3M, A-dec</t>
         </is>
       </c>
       <c r="N24" s="10" t="inlineStr">
         <is>
-          <t>Facebook, Instagram, Twitter/X, YouTube</t>
+          <t>Since 2009</t>
+        </is>
+      </c>
+      <c r="O24" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P24" s="10" t="inlineStr">
+        <is>
+          <t>Facebook, Twitter/X, TikTok</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2460,7 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Pearson Dental Supply Inc</t>
+          <t>Burkhart Dental Supply - Houston</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
@@ -2248,17 +2470,17 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>(713) 690-5111</t>
+          <t>(281) 821-7000</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>http://www.pearsondental.com/</t>
+          <t>http://www.burkhartdental.com/</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>practicesupportteam@burkhartdental.com</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
@@ -2273,32 +2495,42 @@
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>Dental Supplies</t>
+          <t>Burkhart Account</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="K25" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
         </is>
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="M25" s="12" t="inlineStr">
         <is>
-          <t>linkedin.com/company/pearson-dental</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N25" s="12" t="inlineStr">
         <is>
-          <t>Facebook, Instagram, Twitter/X</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O25" s="12" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/burkhart-dental-supply</t>
+        </is>
+      </c>
+      <c r="P25" s="12" t="inlineStr">
+        <is>
+          <t>Facebook, Twitter/X</t>
         </is>
       </c>
     </row>
@@ -2308,67 +2540,77 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Burkhart Dental Supply - Austin</t>
+          <t>Dental Health Products, Inc. (DHP)</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Austin</t>
+          <t>Sugar Land</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>(877) 363-8717</t>
+          <t>(800) 626-2163</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>http://www.burkhartdental.com/</t>
+          <t>https://www.dhpsupply.com/</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>support@dhpsupply.com</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>Burkhart Account</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I26" s="10" t="inlineStr">
         <is>
-          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J26" s="10" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K26" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Dental Supplies, Orthodontic Supplies, Sterilisation, Dental Furniture</t>
         </is>
       </c>
       <c r="L26" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Texas, Southwest, Southeast</t>
         </is>
       </c>
       <c r="M26" s="10" t="inlineStr">
         <is>
-          <t>linkedin.com/company/burkhart-dental-supply</t>
+          <t>3M</t>
         </is>
       </c>
       <c r="N26" s="10" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O26" s="10" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/dhpsupply</t>
+        </is>
+      </c>
+      <c r="P26" s="10" t="inlineStr">
+        <is>
+          <t>Facebook, Instagram, Twitter/X, YouTube</t>
         </is>
       </c>
     </row>
@@ -2378,67 +2620,77 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Burkhart Dental Supply - Houston</t>
+          <t>Dental Creations, Ltd.</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Waco</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>(281) 821-7000</t>
+          <t>(254) 772-4661</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>http://www.burkhartdental.com/</t>
+          <t>https://dentalcreationsltd.com/</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>sales@wonderfill.com</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>Burkhart Account</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H27" s="12" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>Dental Equipment, Dental Supplies, Orthodontic Supplies, Sterilisation</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J27" s="12" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
           <t>Texas</t>
         </is>
       </c>
-      <c r="K27" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L27" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="M27" s="12" t="inlineStr">
         <is>
-          <t>linkedin.com/company/burkhart-dental-supply</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="N27" s="12" t="inlineStr">
         <is>
-          <t>Facebook</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O27" s="12" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/35694029</t>
+        </is>
+      </c>
+      <c r="P27" s="12" t="inlineStr">
+        <is>
+          <t>Facebook, Instagram, YouTube, Google Business</t>
         </is>
       </c>
     </row>
@@ -2448,27 +2700,27 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Dental Creations, Ltd.</t>
+          <t>Garland Dental Equipment Services</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Waco</t>
+          <t>Garland</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>(254) 772-4661</t>
+          <t>(214) 461-5618</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>https://dentalcreationsltd.com/</t>
+          <t>https://www.garlanddental.com/</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>sales@wonderfill.com</t>
+          <t>ecom-swiper@11.css</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -2488,12 +2740,12 @@
       </c>
       <c r="J28" s="10" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="K28" s="10" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Digital Dentistry, Repair &amp; Service</t>
         </is>
       </c>
       <c r="L28" s="10" t="inlineStr">
@@ -2508,14 +2760,24 @@
       </c>
       <c r="N28" s="10" t="inlineStr">
         <is>
-          <t>Facebook, Instagram, YouTube</t>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O28" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P28" s="10" t="inlineStr">
+        <is>
+          <t>Facebook, Instagram</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>